<commit_message>
feat(F-NAR-019): ATOM-EMO.LEX.003-02 Amir, le canard et le miel
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-EMO.LEX.003-02.xlsx
+++ b/stories/arbres/ATOM-EMO.LEX.003-02.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>parc, puis cuisine</t>
+          <t>parc, puis cuisine, kiosque, volet, crochet, herbe, eau, pain, placard, canard, bateau, confiture, miel</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Au parc, le bateau bleu n'est plus là. Amir dit qu'il est déçu. Il choisit un canard en bois. À la cuisine, plus de confiture. Il propose du miel.</t>
+          <t>Une cheville de bois tient le volet. Sur le bois peint, un éclat de kiosque luit. Amir veut le bateau bleu, maintenant. Le crochet est vide. Sourire parti. Papa s'accroupit. Je suis déçu. Merci vécu. Un canard en bois. Deuxième ruse : plus de confiture, le pot glisse. Il refuse de foncer. Il propose le miel. Un éclat de kiosque tient.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>La fontaine laisse tomber des gouttes. L'eau fait un petit cercle, puis plus. Un sac en papier froisse dans la main de papa. L'herbe mouillée colle aux chaussures. Un canard vrai glisse, plus loin. Amir, tu as tes mains dans tes poches ? Oui. Elles sont froides. On reste près de l'eau, d'accord ? D'accord, papa. En ce moment, Amir cherche un bateau bleu. Un petit bateau, pour l'eau. Le bleu, papa. On regarde, oui. Le bateau bleu n'est plus là. Il n'y en a plus. Amir sent ses épaules tomber. Sa gorge se serre. Je suis déçu. Tu es déçu. Ce n'est pas honteux. Un souhait peut attendre. On peut chercher une autre idée. Souffle une fois, Amir. Amir souffle une fois. Il regarde un canard en bois. Celui-là, alors. Le canard. C'est une autre idée. Bravo. Tu as nommé : déçu. Ils prennent le canard. Amir le fait glisser sur l'eau. Le bois est lisse et froid. Il glisse, maman. Il glisse, oui. Plus tard, ils rentrent à la cuisine. La table sent le pain. Une miette reste près du bol. Amir veut de la confiture de fraise. Je regarde le placard. Il n'y en a plus. Amir sent encore les épaules tomber. Je suis déçu. Tu es déçu. Une autre idée. Un souhait peut attendre. Du miel sur le pain. Oui. Du miel. C'est une autre idée. Ils tartinent ensemble. Le miel est collant et doré. Au parc, puis ici, c'est pareil. On nomme : déçu. Puis une autre idée. Le canard, puis le miel. Bravo, Amir. Le miel brille sur le pain.</t>
+          <t>Une cheville de bois tient le volet du kiosque. Elle est coincée, papa. Tu la vois, la cheville ? Oui, papa. La sandale d'Amir tord sa lanière. Elle serre, maman. Tu la lâches, la lanière ? Oui, maman. Papa défait le nœud, près du kiosque. Mes orteils bougent. Ils sont libres, Amir ? Oui. C'est le kiosque des petits bateaux. Des petits bateaux. Tu le vois, le kiosque ? Oui, maman. La peinture du kiosque est tiède, un peu poudreuse. Elle colle un peu. Tu la touches, la peinture ? Oui, papa. Sur le bois peint, un éclat de kiosque luit. Il brille, papa. Tu le vois, le petit point ? Oui, un point clair. Un sac en papier froisse dans la main de maman. Il fait du bruit. Tu l'entends, le papier ? Oui. Une corde pend sous le volet, trop courte. Elle ne touche pas. Tu la vois, la corde ? Oui, papa. Le parc sent l'herbe coupée, près des genoux. Ça sent l'herbe. Tu la sens, l'herbe chaude ? Oui, maman. Un crochet vide attend sous le volet. Il n'a rien. On regarde le crochet ? Oui. En ce moment, Amir cherche un bateau bleu. Le bleu, pour l'eau ! Tout de suite ? Oui, papa. Amir se hausse vers le crochet, trop vite. Sa main trouve du vide. Il n'y en a plus. Le bateau bleu ? Parti. Le sourire d'Amir disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. J'ai mal au ventre. Tu as les épaules lourdes, Amir ? Oui, papa. Papa s'accroupit à la même hauteur. Tes mains sont chaudes, Amir ? Un peu, maman. Je suis déçu. L'éclat de kiosque tremble, puis tient. Tu vois le crochet vide ? Oui. Amir serre les poings, puis les ouvre. Tes poings, Amir ? Ils se desserrent.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>La fontaine laisse tomber des gouttes. L'eau fait un petit cercle, puis plus. Un sac en papier froisse dans la main de papa. L'herbe mouillée colle aux chaussures. Un canard vrai glisse, plus loin. Amir, tu as tes mains dans tes poches ? Oui. Elles sont froides. On reste près de l'eau, d'accord ? D'accord, papa. En ce moment, Amir cherche un bateau bleu. Un petit bateau, pour l'eau. Le bleu, papa. On regarde, oui. Le bateau bleu n'est plus là. Il n'y en a plus. Amir sent ses épaules tomber. Sa gorge se serre. Je suis déçu. Tu es déçu. Ce n'est pas honteux. Un souhait peut attendre. On peut chercher une autre idée. Souffle une fois, Amir. Amir souffle une fois. Il regarde un canard en bois. Celui-là, alors. Le canard. C'est une autre idée. Bravo. Tu as nommé : déçu. Ils prennent le canard. Amir le fait glisser sur l'eau. Le bois est lisse et froid. Il glisse, maman. Il glisse, oui. Plus tard, ils rentrent à la cuisine. La table sent le pain. Une miette reste près du bol. Amir veut de la confiture de fraise. Je regarde le placard. Il n'y en a plus. Amir sent encore les épaules tomber. Je suis déçu. Tu es déçu. Une autre idée. Un souhait peut attendre. Du miel sur le pain. Oui. Du miel. C'est une autre idée. Ils tartinent ensemble. Le miel est collant et doré. Au parc, puis ici, c'est pareil. On nomme : déçu. Puis une autre idée. Le canard, puis le miel. Bravo, Amir. Le miel brille sur le pain.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Une cheville de bois tient le volet du kiosque. Elle est coincée, papa. Tu la vois, la cheville ? Oui, papa. La sandale d'Amir tord sa lanière. Elle serre, maman. Tu la lâches, la lanière ? Oui, maman. Papa défait le nœud, près du kiosque. Mes orteils bougent. Ils sont libres, Amir ? Oui. C'est le kiosque des petits bateaux. Des petits bateaux. Tu le vois, le kiosque ? Oui, maman. La peinture du kiosque est tiède, un peu poudreuse. Elle colle un peu. Tu la touches, la peinture ? Oui, papa. Sur le bois peint, un &lt;emphasis level="moderate"&gt;éclat de kiosque&lt;/emphasis&gt; luit. Il brille, papa. Tu le vois, le petit point ? Oui, un point clair. Un sac en papier froisse dans la main de maman. Il fait du bruit. Tu l'entends, le papier ? Oui. Une corde pend sous le volet, trop courte. Elle ne touche pas. Tu la vois, la corde ? Oui, papa. Le parc sent l'herbe coupée, près des genoux. Ça sent l'herbe. Tu la sens, l'herbe chaude ? Oui, maman. Un crochet vide attend sous le volet. Il n'a rien. On regarde le crochet ? Oui. En ce moment, Amir cherche un bateau bleu. Le bleu, pour l'eau ! Tout de suite ? Oui, papa. Amir se hausse vers le crochet, trop vite. Sa main trouve du vide. Il n'y en a plus. Le bateau bleu ? Parti. Le sourire d'Amir disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. J'ai mal au ventre. Tu as les épaules lourdes, Amir ? Oui, papa. Papa s'accroupit à la même hauteur. Tes mains sont chaudes, Amir ? Un peu, maman. Je suis déçu. L'éclat de kiosque tremble, puis tient. Tu vois le crochet vide ? Oui. Amir serre les poings, puis les ouvre. Tes poings, Amir ? Ils se desserrent.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Ilyes marche au parc. Sa main est dans la main de papa. Il sent l'herbe coupée. Il veut un bateau bleu. Le stand dit : il n'y en a plus. Ilyes sent ses épaules tomber. Sa gorge se serre. Ilyes dit : je suis &lt;emphasis&gt;déçu&lt;/emphasis&gt;. Être déçu, ce n'est pas honteux. Papa s'accroupit. Papa dit : un souhait peut attendre. On peut chercher une autre idée. Ilyes souffle une fois. Il regarde un canard en bois. Il dit : celui-là, alors. Papa sourit. Ils prennent le canard. Ilyes le fait glisser sur l'eau. Plus tard, ils rentrent à la cuisine. Ilyes veut de la confiture de fraise. Maman ouvre le placard. Il n'y en a plus. Ilyes sent encore les épaules tomber. Il dit : je suis déçu. Maman dit : une autre idée. Ilyes propose du miel sur le pain. Maman dit : oui. Ils tartinent ensemble. Le miel est collant. Au parc, puis à la cuisine, c'est pareil. On nomme : déçu. Puis on cherche une autre idée. [pause]</t>
+          <t>Une cheville de bois tient le volet du kiosque. Elle est coincée, papa. Tu la vois, la cheville ? Oui, papa. La sandale d'Amir tord sa lanière. Elle serre, maman. Tu la lâches, la lanière ? Oui, maman. Papa défait le nœud, près du kiosque. Mes orteils bougent. Ils sont libres, Amir ? Oui. C'est le kiosque des petits bateaux. Des petits bateaux. Tu le vois, le kiosque ? Oui, maman. La peinture du kiosque est tiède, un peu poudreuse. Elle colle un peu. Tu la touches, la peinture ? Oui, papa. Sur le bois peint, un &lt;emphasis&gt;éclat de kiosque&lt;/emphasis&gt; luit. Il brille, papa. Tu le vois, le petit point ? Oui, un point clair. Un sac en papier froisse dans la main de maman. Il fait du bruit. Tu l'entends, le papier ? Oui. Une corde pend sous le volet, trop courte. Elle ne touche pas. Tu la vois, la corde ? Oui, papa. Le parc sent l'herbe coupée, près des genoux. Ça sent l'herbe. Tu la sens, l'herbe chaude ? Oui, maman. Un crochet vide attend sous le volet. Il n'a rien. On regarde le crochet ? Oui. En ce moment, Amir cherche un bateau bleu. Le bleu, pour l'eau ! Tout de suite ? Oui, papa. Amir se hausse vers le crochet, trop vite. Sa main trouve du vide. Il n'y en a plus. Le bateau bleu ? Parti. Le sourire d'Amir disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. J'ai mal au ventre. Tu as les épaules lourdes, Amir ? Oui, papa. Papa s'accroupit à la même hauteur. Tes mains sont chaudes, Amir ? Un peu, maman. Je suis déçu. L'éclat de kiosque tremble, puis tient. Tu vois le crochet vide ? Oui. Amir serre les poings, puis les ouvre. Tes poings, Amir ? Ils se desserrent. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,7 +1249,7 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
         <v>1.12</v>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>déçu</t>
+          <t>éclat de kiosque</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,60 +1321,78 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis déception; intensite=2; destinataire=enfant; sous_texte=il_veut_le_bateau_bleu_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|La fontaine laisse tomber des gouttes.
-narrateur|L'eau fait un petit cercle, puis plus.
-narrateur|Un sac en papier froisse dans la main de papa.
-narrateur|L'herbe mouillée colle aux chaussures.
-narrateur|Un canard vrai glisse, plus loin.
-maman|Amir, tu as tes mains dans tes poches ?
-enfant-m|Oui. Elles sont froides.
-papa|On reste près de l'eau, d'accord ?
-enfant-m|D'accord, papa.
+          <t>narrateur|Une cheville de bois tient le volet du kiosque.
+enfant-m|Elle est coincée, papa.
+papa|Tu la vois, la cheville ?
+enfant-m|Oui, papa.
+narrateur|La sandale d'Amir tord sa lanière.
+enfant-m|Elle serre, maman.
+maman|Tu la lâches, la lanière ?
+enfant-m|Oui, maman.
+narrateur|Papa défait le nœud, près du kiosque.
+enfant-m|Mes orteils bougent.
+papa|Ils sont libres, Amir ?
+enfant-m|Oui.
+narrateur|C'est le kiosque des petits bateaux.
+enfant-m|Des petits bateaux.
+maman|Tu le vois, le kiosque ?
+enfant-m|Oui, maman.
+narrateur|La peinture du kiosque est tiède, un peu poudreuse.
+enfant-m|Elle colle un peu.
+papa|Tu la touches, la peinture ?
+enfant-m|Oui, papa.
+narrateur|Sur le bois peint, un éclat de kiosque luit.
+enfant-m|Il brille, papa.
+papa|Tu le vois, le petit point ?
+enfant-m|Oui, un point clair.
+narrateur|Un sac en papier froisse dans la main de maman.
+enfant-m|Il fait du bruit.
+maman|Tu l'entends, le papier ?
+enfant-m|Oui.
+narrateur|Une corde pend sous le volet, trop courte.
+enfant-m|Elle ne touche pas.
+papa|Tu la vois, la corde ?
+enfant-m|Oui, papa.
+narrateur|Le parc sent l'herbe coupée, près des genoux.
+enfant-m|Ça sent l'herbe.
+maman|Tu la sens, l'herbe chaude ?
+enfant-m|Oui, maman.
+narrateur|Un crochet vide attend sous le volet.
+enfant-m|Il n'a rien.
+papa|On regarde le crochet ?
+enfant-m|Oui.
 narrateur|En ce moment, Amir cherche un bateau bleu.
-narrateur|Un petit bateau, pour l'eau.
-enfant-m|Le bleu, papa.
-papa|On regarde, oui.
-narrateur|Le bateau bleu n'est plus là.
+enfant-m|Le bleu, pour l'eau !
+papa|Tout de suite ?
+enfant-m|Oui, papa.
+narrateur|Amir se hausse vers le crochet, trop vite.
+narrateur|Sa main trouve du vide.
 enfant-m|Il n'y en a plus.
-narrateur|Amir sent ses épaules tomber.
-narrateur|Sa gorge se serre.
+maman|Le bateau bleu ?
+enfant-m|Parti.
+narrateur|Le sourire d'Amir disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Ses épaules tombent un peu.
+enfant-m|J'ai mal au ventre.
+papa|Tu as les épaules lourdes, Amir ?
+enfant-m|Oui, papa.
+narrateur|Papa s'accroupit à la même hauteur.
+maman|Tes mains sont chaudes, Amir ?
+enfant-m|Un peu, maman.
 enfant-m|Je suis déçu.
-papa|Tu es déçu. Ce n'est pas honteux.
-papa|Un souhait peut attendre.
-papa|On peut chercher une autre idée.
-maman|Souffle une fois, Amir.
-narrateur|Amir souffle une fois.
-narrateur|Il regarde un canard en bois.
-enfant-m|Celui-là, alors.
-papa|Le canard. C'est une autre idée.
-maman|Bravo. Tu as nommé : déçu.
-narrateur|Ils prennent le canard.
-narrateur|Amir le fait glisser sur l'eau.
-narrateur|Le bois est lisse et froid.
-enfant-m|Il glisse, maman.
-maman|Il glisse, oui.
-narrateur|Plus tard, ils rentrent à la cuisine.
-narrateur|La table sent le pain.
-narrateur|Une miette reste près du bol.
-narrateur|Amir veut de la confiture de fraise.
-maman|Je regarde le placard.
-narrateur|Il n'y en a plus.
-narrateur|Amir sent encore les épaules tomber.
-enfant-m|Je suis déçu.
-maman|Tu es déçu. Une autre idée.
-papa|Un souhait peut attendre.
-enfant-m|Du miel sur le pain.
-maman|Oui. Du miel. C'est une autre idée.
-narrateur|Ils tartinent ensemble.
-narrateur|Le miel est collant et doré.
-papa|Au parc, puis ici, c'est pareil.
-papa|On nomme : déçu. Puis une autre idée.
-enfant-m|Le canard, puis le miel.
-maman|Bravo, Amir.
-narrateur|Le miel brille sur le pain.</t>
+narrateur|L'éclat de kiosque tremble, puis tient.
+papa|Tu vois le crochet vide ?
+enfant-m|Oui.
+narrateur|Amir serre les poings, puis les ouvre.
+papa|Tes poings, Amir ?
+enfant-m|Ils se desserrent.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1411,12 +1429,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Le bateau n'est plus là. Que dit Amir ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Le bateau n'est plus là. Que dit &lt;emphasis level="moderate"&gt;Amir&lt;/emphasis&gt; ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Le bateau n'est plus là. Que dit Ilyes ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Le bateau n'est plus là. Que dit &lt;emphasis&gt;Amir&lt;/emphasis&gt; ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1441,7 +1459,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Ilyes cherche une autre idée. Que dit-il d'abord ?</t>
+          <t>Amir cherche une autre idée. Que dit-il d'abord ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1479,18 +1497,18 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.24</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1505,34 +1523,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Amir</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1541,28 +1563,29 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=le_bateau_n_est_plus_la_que_dit_amir; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Le bateau n'est plus là. Que dit Amir ?</t>
+          <t>narrateur|Le bateau n'est plus là.
+narrateur|Que dit Amir ?</t>
         </is>
       </c>
     </row>
@@ -1589,17 +1612,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Amir tient encore le canard en bois. Je suis déçu. Oui. Et une autre idée est arrivée. Le souhait peut attendre. Bravo. Tu as dit ce que tu sentais. Tu as choisi le canard ? Oui. Puis le miel. Le bois du canard est encore froid. La tartine attend près du bol.</t>
+          <t>Amir avance la main vers le bois, trop vite. Je prends tout, maintenant ! Les mots se bousculent dans sa bouche. N'importe quoi. Amir avance les mains, trop vite. Puis il s'arrête. Amir refuse de foncer. Il referme la bouche. Personne ne parle. Il observe le kiosque, un instant. Il écoute le parc, près du volet. Celui-là. Un canard en bois attend, près du crochet. Tu le prends, Amir ? Oui, le canard. Merci, Amir. Papa reste à la même hauteur. Le bois est froid, sous les doigts. Il est lisse. Ils marchent vers l'eau, sans se presser. Amir pose le canard, tout petit. Il glisse ! Tu le vois, sur l'eau ? Oui, papa. Le bois tient, Amir ? Oui, maman. Le ventre d'Amir se desserre. Les épaules se relèvent un peu. On rentre, après l'eau ? Oui. Amir reprend le canard, sans se bousculer. Il vient avec nous. Tes mains sont au chaud, Amir ? Un peu, maman. La cuisine, plus tard. Oui, papa. Le canard reste contre sa chemise. Il est un peu mouillé.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Amir tient encore le canard en bois. Je suis déçu. Oui. Et une autre idée est arrivée. Le souhait peut attendre. Bravo. Tu as dit ce que tu sentais. Tu as choisi le canard ? Oui. Puis le miel. Le bois du canard est encore froid. La tartine attend près du bol.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir avance la main vers le bois, trop vite. Je prends tout, maintenant ! Les mots se bousculent dans sa bouche. N'importe quoi. Amir avance les mains, trop vite. Puis il s'arrête. Amir refuse de foncer. Il referme la bouche. Personne ne parle. Il observe le kiosque, un instant. Il écoute le parc, près du volet. Celui-là. Un &lt;emphasis level="moderate"&gt;canard&lt;/emphasis&gt; en bois attend, près du crochet. Tu le prends, Amir ? Oui, le canard. Merci, Amir. Papa reste à la même hauteur. Le bois est froid, sous les doigts. Il est lisse. Ils marchent vers l'eau, sans se presser. Amir pose le canard, tout petit. Il glisse ! Tu le vois, sur l'eau ? Oui, papa. Le bois tient, Amir ? Oui, maman. Le ventre d'Amir se desserre. Les épaules se relèvent un peu. On rentre, après l'eau ? Oui. Amir reprend le canard, sans se bousculer. Il vient avec nous. Tes mains sont au chaud, Amir ? Un peu, maman. La cuisine, plus tard. Oui, papa. Le canard reste contre sa chemise. Il est un peu mouillé.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Ilyes a nommé : &lt;emphasis&gt;déçu&lt;/emphasis&gt;. Le souhait peut attendre. Une autre idée est arrivée. [pause]</t>
+          <t>Amir avance la main vers le bois, trop vite. Je prends tout, maintenant ! Les mots se bousculent dans sa bouche. N'importe quoi. Amir avance les mains, trop vite. Puis il s'arrête. Amir refuse de foncer. Il referme la bouche. Personne ne parle. Il observe le kiosque, un instant. Il écoute le parc, près du volet. Celui-là. Un &lt;emphasis&gt;canard&lt;/emphasis&gt; en bois attend, près du crochet. Tu le prends, Amir ? Oui, le canard. Merci, Amir. Papa reste à la même hauteur. Le bois est froid, sous les doigts. Il est lisse. Ils marchent vers l'eau, sans se presser. Amir pose le canard, tout petit. Il glisse ! Tu le vois, sur l'eau ? Oui, papa. Le bois tient, Amir ? Oui, maman. Le ventre d'Amir se desserre. Les épaules se relèvent un peu. On rentre, après l'eau ? Oui. Amir reprend le canard, sans se bousculer. Il vient avec nous. Tes mains sont au chaud, Amir ? Un peu, maman. La cuisine, plus tard. Oui, papa. Le canard reste contre sa chemise. Il est un peu mouillé. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1646,7 +1669,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1654,10 +1677,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.12</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1680,30 +1703,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>déçu</t>
+          <t>canard</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1712,10 +1735,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1728,20 +1751,49 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=il_prend_le_canard_sans_foncer; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Amir tient encore le canard en bois.
-enfant-m|Je suis déçu.
-papa|Oui. Et une autre idée est arrivée.
-maman|Le souhait peut attendre.
-papa|Bravo. Tu as dit ce que tu sentais.
-papa|Tu as choisi le canard ?
-enfant-m|Oui. Puis le miel.
-narrateur|Le bois du canard est encore froid.
-narrateur|La tartine attend près du bol.</t>
+          <t>narrateur|Amir avance la main vers le bois, trop vite.
+enfant-m|Je prends tout, maintenant !
+narrateur|Les mots se bousculent dans sa bouche.
+enfant-m|N'importe quoi.
+narrateur|Amir avance les mains, trop vite.
+narrateur|Puis il s'arrête.
+narrateur|Amir refuse de foncer.
+narrateur|Il referme la bouche.
+narrateur|Personne ne parle.
+narrateur|Il observe le kiosque, un instant.
+narrateur|Il écoute le parc, près du volet.
+enfant-m|Celui-là.
+narrateur|Un canard en bois attend, près du crochet.
+papa|Tu le prends, Amir ?
+enfant-m|Oui, le canard.
+papa|Merci, Amir.
+narrateur|Papa reste à la même hauteur.
+maman|Le bois est froid, sous les doigts.
+enfant-m|Il est lisse.
+narrateur|Ils marchent vers l'eau, sans se presser.
+narrateur|Amir pose le canard, tout petit.
+enfant-m|Il glisse !
+papa|Tu le vois, sur l'eau ?
+enfant-m|Oui, papa.
+maman|Le bois tient, Amir ?
+enfant-m|Oui, maman.
+narrateur|Le ventre d'Amir se desserre.
+narrateur|Les épaules se relèvent un peu.
+papa|On rentre, après l'eau ?
+enfant-m|Oui.
+narrateur|Amir reprend le canard, sans se bousculer.
+enfant-m|Il vient avec nous.
+maman|Tes mains sont au chaud, Amir ?
+enfant-m|Un peu, maman.
+papa|La cuisine, plus tard.
+enfant-m|Oui, papa.
+narrateur|Le canard reste contre sa chemise.
+enfant-m|Il est un peu mouillé.</t>
         </is>
       </c>
     </row>
@@ -1768,17 +1820,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Amir croque la tartine. Le miel colle un peu aux doigts. Le canard repose près du bol. Il me regarde. Tu as encore du miel aux doigts ? Un peu. Tu as trouvé une autre idée. Je suis moins déçu. Le miel est là. Le canard aussi. Ils restent à table, tout calmes.</t>
+          <t>La cuisine sent le pain chaud. Ça sent le pain, maman. Tu le sens, le pain ? Oui. Le canard repose près du pain. De la confiture, maintenant ! Amir ouvre le placard, trop vite. Un pot de fraise tremble, presque vide. Il n'y en a plus. La confiture de fraise ? Parti. Les épaules d'Amir retombent. Je la prends, tout de suite ! Amir avance trop vite vers le pot. Le pot glisse au bord. Il part ! Amir avance les mains, trop vite. Puis il s'arrête net. Amir refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe le placard, un instant. Il écoute la cuisine, près du pain. Sur le bois du canard, un éclat de kiosque luit. Là, sur le bois. On tient le pot ? Oui, papa. Le couvercle du miel résiste, un moment. Le miel, alors. Tu le vois, le pot ? Oui, maman. Papa tourne le couvercle, sans se presser. Le couvercle cède, tout petit. Il s'ouvre ! Ils tartinent le pain, ensemble. Le pain est prêt, Amir ? Oui, papa. Le miel colle un peu au pain. Ça tient.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Amir croque la tartine. Le miel colle un peu aux doigts. Le canard repose près du bol. Il me regarde. Tu as encore du miel aux doigts ? Un peu. Tu as trouvé une autre idée. Je suis moins déçu. Le miel est là. Le canard aussi. Ils restent à table, tout calmes.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La cuisine sent le pain chaud. Ça sent le pain, maman. Tu le sens, le pain ? Oui. Le canard repose près du pain. De la confiture, maintenant ! Amir ouvre le placard, trop vite. Un pot de fraise tremble, presque vide. Il n'y en a plus. La confiture de fraise ? Parti. Les épaules d'Amir retombent. Je la prends, tout de suite ! Amir avance trop vite vers le pot. Le pot glisse au bord. Il part ! Amir avance les mains, trop vite. Puis il s'arrête net. Amir refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe le placard, un instant. Il écoute la cuisine, près du pain. Sur le bois du canard, un &lt;emphasis level="moderate"&gt;éclat de kiosque&lt;/emphasis&gt; luit. Là, sur le bois. On tient le pot ? Oui, papa. Le couvercle du miel résiste, un moment. Le miel, alors. Tu le vois, le pot ? Oui, maman. Papa tourne le couvercle, sans se presser. Le couvercle cède, tout petit. Il s'ouvre ! Ils tartinent le pain, ensemble. Le pain est prêt, Amir ? Oui, papa. Le miel colle un peu au pain. Ça tient.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Ilyes croque la tartine. Le canard repose près du bol. [pause]</t>
+          <t>La cuisine sent le pain chaud. Ça sent le pain, maman. Tu le sens, le pain ? Oui. Le canard repose près du pain. De la confiture, maintenant ! Amir ouvre le placard, trop vite. Un pot de fraise tremble, presque vide. Il n'y en a plus. La confiture de fraise ? Parti. Les épaules d'Amir retombent. Je la prends, tout de suite ! Amir avance trop vite vers le pot. Le pot glisse au bord. Il part ! Amir avance les mains, trop vite. Puis il s'arrête net. Amir refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe le placard, un instant. Il écoute la cuisine, près du pain. Sur le bois du canard, un &lt;emphasis&gt;éclat de kiosque&lt;/emphasis&gt; luit. Là, sur le bois. On tient le pot ? Oui, papa. Le couvercle du miel résiste, un moment. Le miel, alors. Tu le vois, le pot ? Oui, maman. Papa tourne le couvercle, sans se presser. Le couvercle cède, tout petit. Il s'ouvre ! Ils tartinent le pain, ensemble. Le pain est prêt, Amir ? Oui, papa. Le miel colle un peu au pain. Ça tient. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1825,7 +1877,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1833,10 +1885,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.12</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1857,28 +1909,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de kiosque</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1887,10 +1943,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1901,19 +1957,52 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=plus_de_confiture_il_refuse_de_foncer_il_propose_le_miel; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Amir croque la tartine.
-narrateur|Le miel colle un peu aux doigts.
-maman|Le canard repose près du bol.
-enfant-m|Il me regarde.
-maman|Tu as encore du miel aux doigts ?
-enfant-m|Un peu.
-papa|Tu as trouvé une autre idée.
-enfant-m|Je suis moins déçu.
-maman|Le miel est là. Le canard aussi.
-narrateur|Ils restent à table, tout calmes.</t>
+          <t>narrateur|La cuisine sent le pain chaud.
+enfant-m|Ça sent le pain, maman.
+maman|Tu le sens, le pain ?
+enfant-m|Oui.
+narrateur|Le canard repose près du pain.
+enfant-m|De la confiture, maintenant !
+narrateur|Amir ouvre le placard, trop vite.
+narrateur|Un pot de fraise tremble, presque vide.
+enfant-m|Il n'y en a plus.
+maman|La confiture de fraise ?
+enfant-m|Parti.
+narrateur|Les épaules d'Amir retombent.
+enfant-m|Je la prends, tout de suite !
+narrateur|Amir avance trop vite vers le pot.
+narrateur|Le pot glisse au bord.
+enfant-m|Il part !
+narrateur|Amir avance les mains, trop vite.
+narrateur|Puis il s'arrête net.
+narrateur|Amir refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Il observe le placard, un instant.
+narrateur|Il écoute la cuisine, près du pain.
+narrateur|Sur le bois du canard, un éclat de kiosque luit.
+enfant-m|Là, sur le bois.
+papa|On tient le pot ?
+enfant-m|Oui, papa.
+narrateur|Le couvercle du miel résiste, un moment.
+enfant-m|Le miel, alors.
+maman|Tu le vois, le pot ?
+enfant-m|Oui, maman.
+narrateur|Papa tourne le couvercle, sans se presser.
+narrateur|Le couvercle cède, tout petit.
+enfant-m|Il s'ouvre !
+narrateur|Ils tartinent le pain, ensemble.
+papa|Le pain est prêt, Amir ?
+enfant-m|Oui, papa.
+narrateur|Le miel colle un peu au pain.
+enfant-m|Ça tient.</t>
         </is>
       </c>
     </row>
@@ -1940,17 +2029,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit : je suis déçu. J'ai trouvé une autre idée. Un souhait peut attendre. Bravo, Amir.</t>
+          <t>Ils restent près de la table. Maman essuie un peu de pain. Le bateau n'était pas là, papa. Tu l'as vu, toi ? Oui, le crochet vide. On est bien, ici. Amir tapote le canard du doigt. Il a une trace de peinture. Tu la vois, la trace ? Oui, maman. Le canard est resté, Amir. Oui, avec le pain. Ça sent le pain, un peu tiède. Et le bois, maman. Oui, dans l'air. La cuisine est calme, Amir ? Oui, papa. Le canard reste près du pain. Un éclat de kiosque tient sur le bois.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit : je suis déçu. J'ai trouvé une autre idée. Un souhait peut attendre. Bravo, Amir.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près de la table. Maman essuie un peu de pain. Le bateau n'était pas là, papa. Tu l'as vu, toi ? Oui, le crochet vide. On est bien, ici. Amir tapote le canard du doigt. Il a une trace de peinture. Tu la vois, la trace ? Oui, maman. Le canard est resté, Amir. Oui, avec le pain. Ça sent le pain, un peu tiède. Et le bois, maman. Oui, dans l'air. La cuisine est calme, Amir ? Oui, papa. Le canard reste près du pain. Un &lt;emphasis level="moderate"&gt;éclat de kiosque&lt;/emphasis&gt; tient sur le bois.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près de la table. Maman essuie un peu de pain. Le bateau n'était pas là, papa. Tu l'as vu, toi ? Oui, le crochet vide. On est bien, ici. Amir tapote le canard du doigt. Il a une trace de peinture. Tu la vois, la trace ? Oui, maman. Le canard est resté, Amir. Oui, avec le pain. Ça sent le pain, un peu tiède. Et le bois, maman. Oui, dans l'air. La cuisine est calme, Amir ? Oui, papa. Le canard reste près du pain. Un &lt;emphasis&gt;éclat de kiosque&lt;/emphasis&gt; tient sur le bois.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -1997,18 +2086,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.2</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2017,12 +2106,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2031,17 +2120,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de kiosque</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2050,11 +2143,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2063,27 +2156,46 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_bois; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-m|J'ai dit : je suis déçu.
-enfant-m|J'ai trouvé une autre idée.
-papa|Un souhait peut attendre.
-maman|Bravo, Amir.</t>
+          <t>narrateur|Ils restent près de la table.
+narrateur|Maman essuie un peu de pain.
+enfant-m|Le bateau n'était pas là, papa.
+papa|Tu l'as vu, toi ?
+enfant-m|Oui, le crochet vide.
+maman|On est bien, ici.
+narrateur|Amir tapote le canard du doigt.
+enfant-m|Il a une trace de peinture.
+maman|Tu la vois, la trace ?
+enfant-m|Oui, maman.
+papa|Le canard est resté, Amir.
+enfant-m|Oui, avec le pain.
+narrateur|Ça sent le pain, un peu tiède.
+enfant-m|Et le bois, maman.
+maman|Oui, dans l'air.
+papa|La cuisine est calme, Amir ?
+enfant-m|Oui, papa.
+narrateur|Le canard reste près du pain.
+narrateur|Un éclat de kiosque tient sur le bois.</t>
         </is>
       </c>
     </row>
@@ -2104,7 +2216,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2154,6 +2266,13 @@
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>